<commit_message>
Ship the Product Owner's edited quotation master template
Adds the "25 BF Kraft" grade (filling the grade block to A7:G24) and relocates
the GSM surcharge table from A26:C29 to $K$7:$M$10, with CBB+PP's per-layer
VLOOKUP updated to match. Edited by hand on the live template by the Product
Owner; committed unchanged so the deployed /export serves the same workbook.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AvadhootPacks_Quotation_Master_v7.xlsx
+++ b/AvadhootPacks_Quotation_Master_v7.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikun\Desktop\Nikunj Work\ERP\LLM Experiments\Costing\quotation-app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikun\Desktop\Nikunj Work\ERP\LLM Experiments\Costing\Quotation-app-v2\quote-gen-be\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F579EFC8-224C-420F-A070-6464D0E75AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B69EFA-7FCC-477A-B1C3-C9FEAB723EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RATE MASTER" sheetId="1" r:id="rId1"/>
@@ -8356,7 +8356,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="354">
   <si>
     <t>CFB QUOTATION MASTER v7</t>
   </si>
@@ -9498,20 +9498,24 @@
     <t>Calc
 GSM
 (Avg)</t>
+  </si>
+  <si>
+    <t>25 BF Kraft</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="d\-mmm\-yy"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9687,6 +9691,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -9841,10 +9852,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -10085,6 +10097,12 @@
     <xf numFmtId="4" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -10133,14 +10151,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -10406,7 +10422,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E78"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -10415,31 +10431,33 @@
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="12" max="12" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="36.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="101" t="s">
+    <row r="1" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="103" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
     </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="100" t="s">
+    <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="102" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>97</v>
       </c>
@@ -10447,7 +10465,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:17" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>98</v>
       </c>
@@ -10472,8 +10490,26 @@
       <c r="H6" s="81" t="s">
         <v>105</v>
       </c>
+      <c r="K6" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="P6" s="84">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>106</v>
       </c>
@@ -10484,7 +10520,7 @@
         <v>31.5</v>
       </c>
       <c r="D7" s="8">
-        <f t="shared" ref="D7:D23" si="0">C7*$B$4</f>
+        <f t="shared" ref="D7:D24" si="0">C7*$B$4</f>
         <v>0.47249999999999998</v>
       </c>
       <c r="E7" s="7">
@@ -10493,12 +10529,27 @@
       <c r="F7" s="7">
         <v>0</v>
       </c>
-      <c r="G7" s="28">
-        <f t="shared" ref="G7:G23" si="1">C7+D7-E7+F7</f>
+      <c r="G7" s="112">
+        <f t="shared" ref="G7:G24" si="1">C7+D7-E7+F7</f>
         <v>30.9725</v>
       </c>
+      <c r="K7" s="14">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M7" s="15">
+        <v>4</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>156</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
         <v>108</v>
       </c>
@@ -10518,12 +10569,30 @@
       <c r="F8" s="7">
         <v>0</v>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="112">
         <f t="shared" si="1"/>
         <v>31.479999999999997</v>
       </c>
+      <c r="K8" s="17">
+        <v>100</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="M8" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="N8" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="P8" s="83">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>110</v>
       </c>
@@ -10543,12 +10612,30 @@
       <c r="F9" s="7">
         <v>0</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="112">
         <f t="shared" si="1"/>
         <v>33.002499999999998</v>
       </c>
+      <c r="K9" s="14">
+        <v>101</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="M9" s="20">
+        <v>0</v>
+      </c>
+      <c r="N9" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="O9" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="P9" s="82">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="10" t="s">
         <v>112</v>
       </c>
@@ -10568,12 +10655,30 @@
       <c r="F10" s="7">
         <v>0</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="112">
         <f t="shared" si="1"/>
         <v>37.57</v>
       </c>
+      <c r="K10" s="17">
+        <v>201</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="M10" s="21">
+        <v>1</v>
+      </c>
+      <c r="N10" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="P10" s="83">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>114</v>
       </c>
@@ -10593,7 +10698,7 @@
       <c r="F11" s="7">
         <v>0</v>
       </c>
-      <c r="G11" s="28">
+      <c r="G11" s="112">
         <f t="shared" si="1"/>
         <v>39.6</v>
       </c>
@@ -10601,19 +10706,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>118</v>
+    <row r="12" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="5">
+        <v>25</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>353</v>
       </c>
       <c r="C12" s="7">
-        <v>43.5</v>
+        <v>41.25</v>
       </c>
       <c r="D12" s="8">
         <f t="shared" si="0"/>
-        <v>0.65249999999999997</v>
+        <v>0.61875000000000002</v>
       </c>
       <c r="E12" s="7">
         <v>1</v>
@@ -10621,437 +10726,354 @@
       <c r="F12" s="7">
         <v>0</v>
       </c>
-      <c r="G12" s="28">
+      <c r="G12" s="112">
+        <f t="shared" ref="G12" si="2">C12+D12-E12+F12</f>
+        <v>40.868749999999999</v>
+      </c>
+      <c r="H12" s="82"/>
+      <c r="K12" s="100" t="s">
+        <v>163</v>
+      </c>
+      <c r="L12" s="101"/>
+      <c r="M12" s="101"/>
+      <c r="N12" s="101"/>
+      <c r="O12" s="101"/>
+      <c r="P12" s="101"/>
+      <c r="Q12" s="101"/>
+    </row>
+    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="7">
+        <v>43.5</v>
+      </c>
+      <c r="D13" s="8">
+        <f t="shared" si="0"/>
+        <v>0.65249999999999997</v>
+      </c>
+      <c r="E13" s="7">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7">
+        <v>0</v>
+      </c>
+      <c r="G13" s="112">
         <f t="shared" si="1"/>
         <v>43.152500000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="5" t="s">
+    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B14" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C14" s="7">
         <v>51</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D14" s="8">
         <f t="shared" si="0"/>
         <v>0.76500000000000001</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E14" s="7">
         <v>1</v>
       </c>
-      <c r="F13" s="7">
-        <v>0</v>
-      </c>
-      <c r="G13" s="28">
+      <c r="F14" s="7">
+        <v>0</v>
+      </c>
+      <c r="G14" s="112">
         <f t="shared" si="1"/>
         <v>50.765000000000001</v>
       </c>
-      <c r="H13" s="82" t="s">
+      <c r="H14" s="82" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="10" t="s">
+    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B15" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C15" s="7">
         <v>35</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D15" s="8">
         <f t="shared" si="0"/>
         <v>0.52500000000000002</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E15" s="7">
         <v>1</v>
       </c>
-      <c r="F14" s="7">
-        <v>0</v>
-      </c>
-      <c r="G14" s="28">
+      <c r="F15" s="7">
+        <v>0</v>
+      </c>
+      <c r="G15" s="112">
         <f t="shared" si="1"/>
         <v>34.524999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="5" t="s">
+    <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B16" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C16" s="7">
         <v>39.5</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D16" s="8">
         <f t="shared" si="0"/>
         <v>0.59250000000000003</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E16" s="7">
         <v>1</v>
       </c>
-      <c r="F15" s="7">
-        <v>0</v>
-      </c>
-      <c r="G15" s="28">
+      <c r="F16" s="7">
+        <v>0</v>
+      </c>
+      <c r="G16" s="112">
         <f t="shared" si="1"/>
         <v>39.092500000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="10" t="s">
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B17" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C17" s="7">
         <v>41.5</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D17" s="8">
         <f t="shared" si="0"/>
         <v>0.62249999999999994</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E17" s="7">
         <v>1</v>
       </c>
-      <c r="F16" s="7">
-        <v>0</v>
-      </c>
-      <c r="G16" s="28">
+      <c r="F17" s="7">
+        <v>0</v>
+      </c>
+      <c r="G17" s="112">
         <f t="shared" si="1"/>
         <v>41.122500000000002</v>
       </c>
-      <c r="H16" s="83" t="s">
+      <c r="H17" s="83" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="5" t="s">
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B18" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C18" s="7">
         <v>44.5</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D18" s="8">
         <f t="shared" si="0"/>
         <v>0.66749999999999998</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E18" s="7">
         <v>1</v>
       </c>
-      <c r="F17" s="7">
-        <v>0</v>
-      </c>
-      <c r="G17" s="28">
+      <c r="F18" s="7">
+        <v>0</v>
+      </c>
+      <c r="G18" s="112">
         <f t="shared" si="1"/>
         <v>44.167499999999997</v>
       </c>
-      <c r="H17" s="82" t="s">
+      <c r="H18" s="82" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="10" t="s">
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B19" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C19" s="7">
         <v>49</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D19" s="8">
         <f t="shared" si="0"/>
         <v>0.73499999999999999</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E19" s="7">
         <v>1.5</v>
       </c>
-      <c r="F18" s="7">
-        <v>0</v>
-      </c>
-      <c r="G18" s="28">
+      <c r="F19" s="7">
+        <v>0</v>
+      </c>
+      <c r="G19" s="112">
         <f t="shared" si="1"/>
         <v>48.234999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="5" t="s">
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B20" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C20" s="7">
         <v>52</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D20" s="8">
         <f t="shared" si="0"/>
         <v>0.78</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E20" s="7">
         <v>1</v>
       </c>
-      <c r="F19" s="7">
-        <v>0</v>
-      </c>
-      <c r="G19" s="28">
+      <c r="F20" s="7">
+        <v>0</v>
+      </c>
+      <c r="G20" s="112">
         <f t="shared" si="1"/>
         <v>51.78</v>
       </c>
-      <c r="H19" s="82" t="s">
+      <c r="H20" s="82" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="10" t="s">
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B21" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C21" s="7">
         <v>76</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D21" s="8">
         <f t="shared" si="0"/>
         <v>1.1399999999999999</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E21" s="7">
         <v>1</v>
       </c>
-      <c r="F20" s="7">
-        <v>0</v>
-      </c>
-      <c r="G20" s="28">
+      <c r="F21" s="7">
+        <v>0</v>
+      </c>
+      <c r="G21" s="112">
         <f t="shared" si="1"/>
         <v>76.14</v>
       </c>
-      <c r="H20" s="83" t="s">
+      <c r="H21" s="83" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="5" t="s">
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B22" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C22" s="7">
         <v>45</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D22" s="8">
         <f t="shared" si="0"/>
         <v>0.67499999999999993</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E22" s="7">
         <v>1</v>
       </c>
-      <c r="F21" s="7">
-        <v>0</v>
-      </c>
-      <c r="G21" s="28">
+      <c r="F22" s="7">
+        <v>0</v>
+      </c>
+      <c r="G22" s="112">
         <f t="shared" si="1"/>
         <v>44.674999999999997</v>
       </c>
-      <c r="H21" s="82" t="s">
+      <c r="H22" s="82" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="10" t="s">
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B23" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C23" s="7">
         <v>44.5</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D23" s="8">
         <f t="shared" si="0"/>
         <v>0.66749999999999998</v>
       </c>
-      <c r="E22" s="7">
+      <c r="E23" s="7">
         <v>1</v>
       </c>
-      <c r="F22" s="7">
-        <v>0</v>
-      </c>
-      <c r="G22" s="28">
+      <c r="F23" s="7">
+        <v>0</v>
+      </c>
+      <c r="G23" s="112">
         <f t="shared" si="1"/>
         <v>44.167499999999997</v>
       </c>
-      <c r="H22" s="83" t="s">
+      <c r="H23" s="83" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="5" t="s">
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B24" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C24" s="7">
         <v>68</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D24" s="8">
         <f t="shared" si="0"/>
         <v>1.02</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E24" s="7">
         <v>1</v>
       </c>
-      <c r="F23" s="7">
-        <v>0</v>
-      </c>
-      <c r="G23" s="28">
+      <c r="F24" s="7">
+        <v>0</v>
+      </c>
+      <c r="G24" s="112">
         <f t="shared" si="1"/>
         <v>68.02</v>
       </c>
-      <c r="H23" s="82" t="s">
+      <c r="H24" s="82" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="F25" s="84">
-        <v>0</v>
-      </c>
-      <c r="G25" s="84" t="e">
-        <f>C25+D25-E25+F25</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="14">
-        <v>0</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="C26" s="15">
-        <v>4</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="17">
-        <v>100</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="C27" s="18">
-        <v>1.5</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="F27" s="83">
-        <v>0</v>
-      </c>
-      <c r="G27" s="83" t="e">
-        <f>C27+D27-E27+F27</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="14">
-        <v>101</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C28" s="20">
-        <v>0</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="F28" s="82">
-        <v>0</v>
-      </c>
-      <c r="G28" s="82" t="e">
-        <f>C28+D28-E28+F28</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="17">
-        <v>201</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="C29" s="21">
-        <v>1</v>
-      </c>
-      <c r="D29" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="F29" s="83">
-        <v>0</v>
-      </c>
-      <c r="G29" s="83" t="e">
-        <f>C29+D29-E29+F29</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="98" t="s">
-        <v>163</v>
-      </c>
-      <c r="B31" s="99"/>
-      <c r="C31" s="99"/>
-      <c r="D31" s="99"/>
-      <c r="E31" s="99"/>
-      <c r="F31" s="99"/>
-      <c r="G31" s="99"/>
-    </row>
+    <row r="26" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="27" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="28" spans="1:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="29" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="30" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="K12:Q12"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -11085,41 +11107,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="105" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="M1" s="104" t="s">
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
+      <c r="K1" s="101"/>
+      <c r="M1" s="106" t="s">
         <v>165</v>
       </c>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
     </row>
     <row r="2" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="100" t="s">
+      <c r="A2" s="102" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="101"/>
+      <c r="I2" s="101"/>
+      <c r="J2" s="101"/>
+      <c r="K2" s="101"/>
       <c r="M2" s="22" t="s">
         <v>167</v>
       </c>
@@ -11135,11 +11157,11 @@
       <c r="Q2" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="T2" s="102" t="s">
+      <c r="T2" s="104" t="s">
         <v>172</v>
       </c>
-      <c r="U2" s="89"/>
-      <c r="V2" s="90"/>
+      <c r="U2" s="91"/>
+      <c r="V2" s="92"/>
     </row>
     <row r="3" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="M3" s="5" t="s">
@@ -11390,13 +11412,13 @@
       <c r="K7" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="M7" s="106" t="s">
+      <c r="M7" s="108" t="s">
         <v>207</v>
       </c>
-      <c r="N7" s="99"/>
-      <c r="O7" s="99"/>
-      <c r="P7" s="99"/>
-      <c r="Q7" s="99"/>
+      <c r="N7" s="101"/>
+      <c r="O7" s="101"/>
+      <c r="P7" s="101"/>
+      <c r="Q7" s="101"/>
       <c r="S7" s="25" t="s">
         <v>169</v>
       </c>
@@ -12101,19 +12123,19 @@
       </c>
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="105" t="s">
+      <c r="A27" s="107" t="s">
         <v>279</v>
       </c>
-      <c r="B27" s="99"/>
-      <c r="C27" s="99"/>
-      <c r="D27" s="99"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="99"/>
-      <c r="G27" s="99"/>
-      <c r="H27" s="99"/>
-      <c r="I27" s="99"/>
-      <c r="J27" s="99"/>
-      <c r="K27" s="99"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
     </row>
     <row r="28" spans="1:22" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="34" t="s">
@@ -12723,98 +12745,98 @@
       </c>
     </row>
     <row r="5" spans="1:72" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="91" t="s">
+      <c r="A5" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="89"/>
-      <c r="C5" s="89"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="89"/>
-      <c r="F5" s="91" t="s">
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="89"/>
-      <c r="H5" s="89"/>
-      <c r="I5" s="92" t="s">
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="89"/>
-      <c r="K5" s="89"/>
-      <c r="L5" s="92" t="s">
+      <c r="J5" s="91"/>
+      <c r="K5" s="91"/>
+      <c r="L5" s="94" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="89"/>
-      <c r="N5" s="89"/>
-      <c r="O5" s="89"/>
-      <c r="P5" s="92" t="s">
+      <c r="M5" s="91"/>
+      <c r="N5" s="91"/>
+      <c r="O5" s="91"/>
+      <c r="P5" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="89"/>
-      <c r="R5" s="89"/>
-      <c r="S5" s="93" t="s">
+      <c r="Q5" s="91"/>
+      <c r="R5" s="91"/>
+      <c r="S5" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="T5" s="96"/>
-      <c r="U5" s="96"/>
-      <c r="V5" s="96"/>
-      <c r="W5" s="96"/>
-      <c r="X5" s="96"/>
-      <c r="Y5" s="96"/>
-      <c r="Z5" s="96"/>
-      <c r="AA5" s="97"/>
-      <c r="AB5" s="95" t="s">
+      <c r="T5" s="98"/>
+      <c r="U5" s="98"/>
+      <c r="V5" s="98"/>
+      <c r="W5" s="98"/>
+      <c r="X5" s="98"/>
+      <c r="Y5" s="98"/>
+      <c r="Z5" s="98"/>
+      <c r="AA5" s="99"/>
+      <c r="AB5" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="AC5" s="89"/>
-      <c r="AD5" s="95" t="s">
+      <c r="AC5" s="91"/>
+      <c r="AD5" s="97" t="s">
         <v>19</v>
       </c>
-      <c r="AE5" s="89"/>
-      <c r="AF5" s="89"/>
-      <c r="AG5" s="89"/>
-      <c r="AH5" s="89"/>
-      <c r="AI5" s="89"/>
-      <c r="AJ5" s="89"/>
-      <c r="AK5" s="89"/>
-      <c r="AL5" s="89"/>
-      <c r="AM5" s="89"/>
-      <c r="AN5" s="93" t="s">
+      <c r="AE5" s="91"/>
+      <c r="AF5" s="91"/>
+      <c r="AG5" s="91"/>
+      <c r="AH5" s="91"/>
+      <c r="AI5" s="91"/>
+      <c r="AJ5" s="91"/>
+      <c r="AK5" s="91"/>
+      <c r="AL5" s="91"/>
+      <c r="AM5" s="91"/>
+      <c r="AN5" s="95" t="s">
         <v>20</v>
       </c>
-      <c r="AO5" s="89"/>
-      <c r="AP5" s="89"/>
-      <c r="AQ5" s="89"/>
-      <c r="AR5" s="89"/>
-      <c r="AS5" s="92" t="s">
+      <c r="AO5" s="91"/>
+      <c r="AP5" s="91"/>
+      <c r="AQ5" s="91"/>
+      <c r="AR5" s="91"/>
+      <c r="AS5" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="AT5" s="89"/>
-      <c r="AU5" s="89"/>
-      <c r="AV5" s="89"/>
-      <c r="AW5" s="89"/>
-      <c r="AX5" s="89"/>
+      <c r="AT5" s="91"/>
+      <c r="AU5" s="91"/>
+      <c r="AV5" s="91"/>
+      <c r="AW5" s="91"/>
+      <c r="AX5" s="91"/>
       <c r="AY5" s="2"/>
-      <c r="AZ5" s="88" t="s">
+      <c r="AZ5" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="BA5" s="89"/>
-      <c r="BB5" s="89"/>
-      <c r="BC5" s="89"/>
-      <c r="BD5" s="89"/>
-      <c r="BE5" s="89"/>
-      <c r="BF5" s="89"/>
-      <c r="BG5" s="89"/>
-      <c r="BH5" s="89"/>
-      <c r="BI5" s="89"/>
-      <c r="BJ5" s="89"/>
-      <c r="BK5" s="90"/>
+      <c r="BA5" s="91"/>
+      <c r="BB5" s="91"/>
+      <c r="BC5" s="91"/>
+      <c r="BD5" s="91"/>
+      <c r="BE5" s="91"/>
+      <c r="BF5" s="91"/>
+      <c r="BG5" s="91"/>
+      <c r="BH5" s="91"/>
+      <c r="BI5" s="91"/>
+      <c r="BJ5" s="91"/>
+      <c r="BK5" s="92"/>
       <c r="BL5" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="BM5" s="94" t="s">
+      <c r="BM5" s="96" t="s">
         <v>24</v>
       </c>
-      <c r="BN5" s="89"/>
+      <c r="BN5" s="91"/>
       <c r="BO5" s="43" t="s">
         <v>25</v>
       </c>
@@ -13118,25 +13140,25 @@
       <c r="AK7" s="28"/>
       <c r="AL7" s="28"/>
       <c r="AM7" s="28"/>
-      <c r="AN7" s="60">
-        <f>IFERROR(VLOOKUP(AD7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE7,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO7" s="60">
-        <f>IFERROR(VLOOKUP(AF7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG7,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP7" s="60">
-        <f>IFERROR(VLOOKUP(AH7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI7,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ7" s="60">
-        <f>IFERROR(VLOOKUP(AJ7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK7,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR7" s="60">
-        <f>IFERROR(VLOOKUP(AL7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM7,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN7" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE7,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO7" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG7,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP7" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI7,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ7" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK7,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR7" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL7,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM7,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS7" s="61">
         <f>IFERROR((AE7/1000)*R7*1*(1+IF(B7="Box",$AY$3,$AY$4)),0)</f>
@@ -13303,25 +13325,25 @@
       <c r="AK8" s="28"/>
       <c r="AL8" s="28"/>
       <c r="AM8" s="28"/>
-      <c r="AN8" s="60">
-        <f>IFERROR(VLOOKUP(AD8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE8,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO8" s="60">
-        <f>IFERROR(VLOOKUP(AF8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG8,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP8" s="60">
-        <f>IFERROR(VLOOKUP(AH8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI8,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ8" s="60">
-        <f>IFERROR(VLOOKUP(AJ8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK8,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR8" s="60">
-        <f>IFERROR(VLOOKUP(AL8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM8,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN8" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE8,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO8" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG8,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP8" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI8,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ8" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK8,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR8" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL8,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM8,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS8" s="61">
         <f t="shared" ref="AS8:AS50" si="17">IFERROR((AE8/1000)*R8*1*(1+IF(B8="Box",$AY$3,$AY$4)),0)</f>
@@ -13488,25 +13510,25 @@
       <c r="AK9" s="28"/>
       <c r="AL9" s="28"/>
       <c r="AM9" s="28"/>
-      <c r="AN9" s="60">
-        <f>IFERROR(VLOOKUP(AD9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE9,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO9" s="60">
-        <f>IFERROR(VLOOKUP(AF9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG9,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP9" s="60">
-        <f>IFERROR(VLOOKUP(AH9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI9,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ9" s="60">
-        <f>IFERROR(VLOOKUP(AJ9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK9,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR9" s="60">
-        <f>IFERROR(VLOOKUP(AL9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM9,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN9" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE9,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO9" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG9,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP9" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI9,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ9" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK9,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR9" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL9,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM9,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS9" s="61">
         <f t="shared" si="17"/>
@@ -13673,25 +13695,25 @@
       <c r="AK10" s="28"/>
       <c r="AL10" s="28"/>
       <c r="AM10" s="28"/>
-      <c r="AN10" s="60">
-        <f>IFERROR(VLOOKUP(AD10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE10,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO10" s="60">
-        <f>IFERROR(VLOOKUP(AF10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG10,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP10" s="60">
-        <f>IFERROR(VLOOKUP(AH10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI10,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ10" s="60">
-        <f>IFERROR(VLOOKUP(AJ10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK10,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR10" s="60">
-        <f>IFERROR(VLOOKUP(AL10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM10,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN10" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE10,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO10" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG10,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP10" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI10,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ10" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK10,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR10" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL10,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM10,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS10" s="61">
         <f t="shared" si="17"/>
@@ -13858,25 +13880,25 @@
       <c r="AK11" s="28"/>
       <c r="AL11" s="28"/>
       <c r="AM11" s="28"/>
-      <c r="AN11" s="60">
-        <f>IFERROR(VLOOKUP(AD11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE11,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO11" s="60">
-        <f>IFERROR(VLOOKUP(AF11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG11,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP11" s="60">
-        <f>IFERROR(VLOOKUP(AH11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI11,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ11" s="60">
-        <f>IFERROR(VLOOKUP(AJ11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK11,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR11" s="60">
-        <f>IFERROR(VLOOKUP(AL11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM11,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN11" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE11,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO11" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG11,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP11" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI11,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ11" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK11,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR11" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL11,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM11,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS11" s="61">
         <f t="shared" si="17"/>
@@ -14043,25 +14065,25 @@
       <c r="AK12" s="28"/>
       <c r="AL12" s="28"/>
       <c r="AM12" s="28"/>
-      <c r="AN12" s="60">
-        <f>IFERROR(VLOOKUP(AD12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE12,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO12" s="60">
-        <f>IFERROR(VLOOKUP(AF12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG12,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP12" s="60">
-        <f>IFERROR(VLOOKUP(AH12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI12,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ12" s="60">
-        <f>IFERROR(VLOOKUP(AJ12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK12,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR12" s="60">
-        <f>IFERROR(VLOOKUP(AL12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM12,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN12" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE12,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO12" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG12,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP12" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI12,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ12" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK12,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR12" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL12,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM12,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS12" s="61">
         <f t="shared" si="17"/>
@@ -14228,25 +14250,25 @@
       <c r="AK13" s="28"/>
       <c r="AL13" s="28"/>
       <c r="AM13" s="28"/>
-      <c r="AN13" s="60">
-        <f>IFERROR(VLOOKUP(AD13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE13,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO13" s="60">
-        <f>IFERROR(VLOOKUP(AF13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG13,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP13" s="60">
-        <f>IFERROR(VLOOKUP(AH13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI13,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ13" s="60">
-        <f>IFERROR(VLOOKUP(AJ13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK13,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR13" s="60">
-        <f>IFERROR(VLOOKUP(AL13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM13,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN13" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE13,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO13" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG13,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP13" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI13,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ13" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK13,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR13" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL13,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM13,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS13" s="61">
         <f t="shared" si="17"/>
@@ -14413,25 +14435,25 @@
       <c r="AK14" s="28"/>
       <c r="AL14" s="28"/>
       <c r="AM14" s="28"/>
-      <c r="AN14" s="60">
-        <f>IFERROR(VLOOKUP(AD14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE14,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO14" s="60">
-        <f>IFERROR(VLOOKUP(AF14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG14,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP14" s="60">
-        <f>IFERROR(VLOOKUP(AH14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI14,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ14" s="60">
-        <f>IFERROR(VLOOKUP(AJ14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK14,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR14" s="60">
-        <f>IFERROR(VLOOKUP(AL14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM14,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN14" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE14,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO14" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG14,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP14" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI14,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ14" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK14,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR14" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL14,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM14,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS14" s="61">
         <f t="shared" si="17"/>
@@ -14598,25 +14620,25 @@
       <c r="AK15" s="28"/>
       <c r="AL15" s="28"/>
       <c r="AM15" s="28"/>
-      <c r="AN15" s="60">
-        <f>IFERROR(VLOOKUP(AD15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE15,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO15" s="60">
-        <f>IFERROR(VLOOKUP(AF15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG15,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP15" s="60">
-        <f>IFERROR(VLOOKUP(AH15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI15,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ15" s="60">
-        <f>IFERROR(VLOOKUP(AJ15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK15,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR15" s="60">
-        <f>IFERROR(VLOOKUP(AL15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM15,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN15" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE15,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO15" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG15,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP15" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI15,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ15" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK15,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR15" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL15,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM15,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS15" s="61">
         <f t="shared" si="17"/>
@@ -14783,25 +14805,25 @@
       <c r="AK16" s="28"/>
       <c r="AL16" s="28"/>
       <c r="AM16" s="28"/>
-      <c r="AN16" s="60">
-        <f>IFERROR(VLOOKUP(AD16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE16,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO16" s="60">
-        <f>IFERROR(VLOOKUP(AF16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG16,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP16" s="60">
-        <f>IFERROR(VLOOKUP(AH16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI16,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ16" s="60">
-        <f>IFERROR(VLOOKUP(AJ16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK16,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR16" s="60">
-        <f>IFERROR(VLOOKUP(AL16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM16,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN16" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE16,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO16" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG16,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP16" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI16,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ16" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK16,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR16" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL16,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM16,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS16" s="61">
         <f t="shared" si="17"/>
@@ -14968,25 +14990,25 @@
       <c r="AK17" s="28"/>
       <c r="AL17" s="28"/>
       <c r="AM17" s="28"/>
-      <c r="AN17" s="60">
-        <f>IFERROR(VLOOKUP(AD17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE17,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO17" s="60">
-        <f>IFERROR(VLOOKUP(AF17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG17,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP17" s="60">
-        <f>IFERROR(VLOOKUP(AH17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI17,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ17" s="60">
-        <f>IFERROR(VLOOKUP(AJ17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK17,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR17" s="60">
-        <f>IFERROR(VLOOKUP(AL17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM17,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN17" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE17,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO17" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG17,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP17" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI17,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ17" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK17,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR17" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL17,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM17,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS17" s="61">
         <f t="shared" si="17"/>
@@ -15153,25 +15175,25 @@
       <c r="AK18" s="28"/>
       <c r="AL18" s="28"/>
       <c r="AM18" s="28"/>
-      <c r="AN18" s="60">
-        <f>IFERROR(VLOOKUP(AD18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE18,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO18" s="60">
-        <f>IFERROR(VLOOKUP(AF18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG18,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP18" s="60">
-        <f>IFERROR(VLOOKUP(AH18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI18,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ18" s="60">
-        <f>IFERROR(VLOOKUP(AJ18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK18,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR18" s="60">
-        <f>IFERROR(VLOOKUP(AL18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM18,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN18" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE18,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO18" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG18,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP18" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI18,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ18" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK18,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR18" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL18,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM18,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS18" s="61">
         <f t="shared" si="17"/>
@@ -15338,25 +15360,25 @@
       <c r="AK19" s="28"/>
       <c r="AL19" s="28"/>
       <c r="AM19" s="28"/>
-      <c r="AN19" s="60">
-        <f>IFERROR(VLOOKUP(AD19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE19,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO19" s="60">
-        <f>IFERROR(VLOOKUP(AF19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG19,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP19" s="60">
-        <f>IFERROR(VLOOKUP(AH19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI19,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ19" s="60">
-        <f>IFERROR(VLOOKUP(AJ19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK19,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR19" s="60">
-        <f>IFERROR(VLOOKUP(AL19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM19,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN19" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE19,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO19" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG19,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP19" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI19,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ19" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK19,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR19" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL19,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM19,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS19" s="61">
         <f t="shared" si="17"/>
@@ -15523,25 +15545,25 @@
       <c r="AK20" s="28"/>
       <c r="AL20" s="28"/>
       <c r="AM20" s="28"/>
-      <c r="AN20" s="60">
-        <f>IFERROR(VLOOKUP(AD20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE20,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO20" s="60">
-        <f>IFERROR(VLOOKUP(AF20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG20,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP20" s="60">
-        <f>IFERROR(VLOOKUP(AH20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI20,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ20" s="60">
-        <f>IFERROR(VLOOKUP(AJ20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK20,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR20" s="60">
-        <f>IFERROR(VLOOKUP(AL20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM20,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN20" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE20,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO20" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG20,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP20" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI20,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ20" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK20,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR20" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL20,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM20,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS20" s="61">
         <f t="shared" si="17"/>
@@ -15708,25 +15730,25 @@
       <c r="AK21" s="28"/>
       <c r="AL21" s="28"/>
       <c r="AM21" s="28"/>
-      <c r="AN21" s="60">
-        <f>IFERROR(VLOOKUP(AD21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE21,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO21" s="60">
-        <f>IFERROR(VLOOKUP(AF21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG21,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP21" s="60">
-        <f>IFERROR(VLOOKUP(AH21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI21,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ21" s="60">
-        <f>IFERROR(VLOOKUP(AJ21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK21,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR21" s="60">
-        <f>IFERROR(VLOOKUP(AL21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM21,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN21" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE21,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO21" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG21,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP21" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI21,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ21" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK21,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR21" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL21,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM21,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS21" s="61">
         <f t="shared" si="17"/>
@@ -15893,25 +15915,25 @@
       <c r="AK22" s="28"/>
       <c r="AL22" s="28"/>
       <c r="AM22" s="28"/>
-      <c r="AN22" s="60">
-        <f>IFERROR(VLOOKUP(AD22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE22,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO22" s="60">
-        <f>IFERROR(VLOOKUP(AF22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG22,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP22" s="60">
-        <f>IFERROR(VLOOKUP(AH22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI22,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ22" s="60">
-        <f>IFERROR(VLOOKUP(AJ22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK22,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR22" s="60">
-        <f>IFERROR(VLOOKUP(AL22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM22,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN22" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE22,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO22" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG22,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP22" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI22,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ22" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK22,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR22" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL22,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM22,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS22" s="61">
         <f t="shared" si="17"/>
@@ -16078,25 +16100,25 @@
       <c r="AK23" s="28"/>
       <c r="AL23" s="28"/>
       <c r="AM23" s="28"/>
-      <c r="AN23" s="60">
-        <f>IFERROR(VLOOKUP(AD23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE23,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO23" s="60">
-        <f>IFERROR(VLOOKUP(AF23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG23,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP23" s="60">
-        <f>IFERROR(VLOOKUP(AH23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI23,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ23" s="60">
-        <f>IFERROR(VLOOKUP(AJ23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK23,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR23" s="60">
-        <f>IFERROR(VLOOKUP(AL23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM23,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN23" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE23,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO23" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG23,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP23" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI23,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ23" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK23,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR23" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL23,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM23,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS23" s="61">
         <f t="shared" si="17"/>
@@ -16263,25 +16285,25 @@
       <c r="AK24" s="28"/>
       <c r="AL24" s="28"/>
       <c r="AM24" s="28"/>
-      <c r="AN24" s="60">
-        <f>IFERROR(VLOOKUP(AD24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE24,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO24" s="60">
-        <f>IFERROR(VLOOKUP(AF24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG24,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP24" s="60">
-        <f>IFERROR(VLOOKUP(AH24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI24,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ24" s="60">
-        <f>IFERROR(VLOOKUP(AJ24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK24,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR24" s="60">
-        <f>IFERROR(VLOOKUP(AL24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM24,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN24" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE24,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO24" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG24,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP24" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI24,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ24" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK24,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR24" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL24,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM24,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS24" s="61">
         <f t="shared" si="17"/>
@@ -16448,25 +16470,25 @@
       <c r="AK25" s="28"/>
       <c r="AL25" s="28"/>
       <c r="AM25" s="28"/>
-      <c r="AN25" s="60">
-        <f>IFERROR(VLOOKUP(AD25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE25,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO25" s="60">
-        <f>IFERROR(VLOOKUP(AF25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG25,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP25" s="60">
-        <f>IFERROR(VLOOKUP(AH25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI25,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ25" s="60">
-        <f>IFERROR(VLOOKUP(AJ25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK25,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR25" s="60">
-        <f>IFERROR(VLOOKUP(AL25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM25,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN25" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE25,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO25" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG25,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP25" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI25,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ25" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK25,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR25" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL25,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM25,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS25" s="61">
         <f t="shared" si="17"/>
@@ -16633,25 +16655,25 @@
       <c r="AK26" s="28"/>
       <c r="AL26" s="28"/>
       <c r="AM26" s="28"/>
-      <c r="AN26" s="60">
-        <f>IFERROR(VLOOKUP(AD26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE26,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO26" s="60">
-        <f>IFERROR(VLOOKUP(AF26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG26,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP26" s="60">
-        <f>IFERROR(VLOOKUP(AH26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI26,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ26" s="60">
-        <f>IFERROR(VLOOKUP(AJ26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK26,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR26" s="60">
-        <f>IFERROR(VLOOKUP(AL26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM26,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN26" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE26,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO26" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG26,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP26" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI26,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ26" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK26,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR26" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL26,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM26,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS26" s="61">
         <f t="shared" si="17"/>
@@ -16818,25 +16840,25 @@
       <c r="AK27" s="28"/>
       <c r="AL27" s="28"/>
       <c r="AM27" s="28"/>
-      <c r="AN27" s="60">
-        <f>IFERROR(VLOOKUP(AD27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE27,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO27" s="60">
-        <f>IFERROR(VLOOKUP(AF27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG27,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP27" s="60">
-        <f>IFERROR(VLOOKUP(AH27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI27,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ27" s="60">
-        <f>IFERROR(VLOOKUP(AJ27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK27,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR27" s="60">
-        <f>IFERROR(VLOOKUP(AL27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM27,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN27" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE27,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO27" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG27,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP27" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI27,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ27" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK27,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR27" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL27,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM27,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS27" s="61">
         <f t="shared" si="17"/>
@@ -17003,25 +17025,25 @@
       <c r="AK28" s="28"/>
       <c r="AL28" s="28"/>
       <c r="AM28" s="28"/>
-      <c r="AN28" s="60">
-        <f>IFERROR(VLOOKUP(AD28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE28,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO28" s="60">
-        <f>IFERROR(VLOOKUP(AF28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG28,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP28" s="60">
-        <f>IFERROR(VLOOKUP(AH28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI28,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ28" s="60">
-        <f>IFERROR(VLOOKUP(AJ28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK28,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR28" s="60">
-        <f>IFERROR(VLOOKUP(AL28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM28,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN28" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE28,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO28" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG28,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP28" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI28,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ28" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK28,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR28" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL28,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM28,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS28" s="61">
         <f t="shared" si="17"/>
@@ -17188,25 +17210,25 @@
       <c r="AK29" s="28"/>
       <c r="AL29" s="28"/>
       <c r="AM29" s="28"/>
-      <c r="AN29" s="60">
-        <f>IFERROR(VLOOKUP(AD29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE29,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO29" s="60">
-        <f>IFERROR(VLOOKUP(AF29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG29,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP29" s="60">
-        <f>IFERROR(VLOOKUP(AH29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI29,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ29" s="60">
-        <f>IFERROR(VLOOKUP(AJ29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK29,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR29" s="60">
-        <f>IFERROR(VLOOKUP(AL29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM29,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN29" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE29,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO29" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG29,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP29" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI29,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ29" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK29,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR29" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL29,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM29,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS29" s="61">
         <f t="shared" si="17"/>
@@ -17373,25 +17395,25 @@
       <c r="AK30" s="28"/>
       <c r="AL30" s="28"/>
       <c r="AM30" s="28"/>
-      <c r="AN30" s="60">
-        <f>IFERROR(VLOOKUP(AD30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE30,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO30" s="60">
-        <f>IFERROR(VLOOKUP(AF30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG30,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP30" s="60">
-        <f>IFERROR(VLOOKUP(AH30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI30,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ30" s="60">
-        <f>IFERROR(VLOOKUP(AJ30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK30,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR30" s="60">
-        <f>IFERROR(VLOOKUP(AL30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM30,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN30" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE30,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO30" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG30,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP30" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI30,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ30" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK30,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR30" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL30,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM30,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS30" s="61">
         <f t="shared" si="17"/>
@@ -17558,25 +17580,25 @@
       <c r="AK31" s="28"/>
       <c r="AL31" s="28"/>
       <c r="AM31" s="28"/>
-      <c r="AN31" s="60">
-        <f>IFERROR(VLOOKUP(AD31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE31,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO31" s="60">
-        <f>IFERROR(VLOOKUP(AF31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG31,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP31" s="60">
-        <f>IFERROR(VLOOKUP(AH31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI31,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ31" s="60">
-        <f>IFERROR(VLOOKUP(AJ31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK31,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR31" s="60">
-        <f>IFERROR(VLOOKUP(AL31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM31,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN31" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE31,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO31" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG31,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP31" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI31,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ31" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK31,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR31" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL31,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM31,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS31" s="61">
         <f t="shared" si="17"/>
@@ -17743,25 +17765,25 @@
       <c r="AK32" s="28"/>
       <c r="AL32" s="28"/>
       <c r="AM32" s="28"/>
-      <c r="AN32" s="60">
-        <f>IFERROR(VLOOKUP(AD32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE32,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO32" s="60">
-        <f>IFERROR(VLOOKUP(AF32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG32,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP32" s="60">
-        <f>IFERROR(VLOOKUP(AH32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI32,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ32" s="60">
-        <f>IFERROR(VLOOKUP(AJ32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK32,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR32" s="60">
-        <f>IFERROR(VLOOKUP(AL32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM32,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN32" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE32,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO32" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG32,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP32" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI32,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ32" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK32,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR32" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL32,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM32,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS32" s="61">
         <f t="shared" si="17"/>
@@ -17928,25 +17950,25 @@
       <c r="AK33" s="28"/>
       <c r="AL33" s="28"/>
       <c r="AM33" s="28"/>
-      <c r="AN33" s="60">
-        <f>IFERROR(VLOOKUP(AD33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE33,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO33" s="60">
-        <f>IFERROR(VLOOKUP(AF33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG33,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP33" s="60">
-        <f>IFERROR(VLOOKUP(AH33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI33,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ33" s="60">
-        <f>IFERROR(VLOOKUP(AJ33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK33,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR33" s="60">
-        <f>IFERROR(VLOOKUP(AL33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM33,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN33" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE33,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO33" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG33,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP33" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI33,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ33" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK33,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR33" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL33,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM33,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS33" s="61">
         <f t="shared" si="17"/>
@@ -18113,25 +18135,25 @@
       <c r="AK34" s="28"/>
       <c r="AL34" s="28"/>
       <c r="AM34" s="28"/>
-      <c r="AN34" s="60">
-        <f>IFERROR(VLOOKUP(AD34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE34,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO34" s="60">
-        <f>IFERROR(VLOOKUP(AF34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG34,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP34" s="60">
-        <f>IFERROR(VLOOKUP(AH34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI34,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ34" s="60">
-        <f>IFERROR(VLOOKUP(AJ34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK34,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR34" s="60">
-        <f>IFERROR(VLOOKUP(AL34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM34,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN34" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE34,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO34" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG34,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP34" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI34,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ34" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK34,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR34" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL34,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM34,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS34" s="61">
         <f t="shared" si="17"/>
@@ -18298,25 +18320,25 @@
       <c r="AK35" s="28"/>
       <c r="AL35" s="28"/>
       <c r="AM35" s="28"/>
-      <c r="AN35" s="60">
-        <f>IFERROR(VLOOKUP(AD35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE35,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO35" s="60">
-        <f>IFERROR(VLOOKUP(AF35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG35,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP35" s="60">
-        <f>IFERROR(VLOOKUP(AH35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI35,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ35" s="60">
-        <f>IFERROR(VLOOKUP(AJ35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK35,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR35" s="60">
-        <f>IFERROR(VLOOKUP(AL35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM35,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN35" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE35,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO35" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG35,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP35" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI35,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ35" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK35,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR35" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL35,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM35,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS35" s="61">
         <f t="shared" si="17"/>
@@ -18483,25 +18505,25 @@
       <c r="AK36" s="28"/>
       <c r="AL36" s="28"/>
       <c r="AM36" s="28"/>
-      <c r="AN36" s="60">
-        <f>IFERROR(VLOOKUP(AD36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE36,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO36" s="60">
-        <f>IFERROR(VLOOKUP(AF36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG36,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP36" s="60">
-        <f>IFERROR(VLOOKUP(AH36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI36,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ36" s="60">
-        <f>IFERROR(VLOOKUP(AJ36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK36,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR36" s="60">
-        <f>IFERROR(VLOOKUP(AL36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM36,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN36" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE36,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO36" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG36,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP36" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI36,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ36" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK36,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR36" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL36,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM36,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS36" s="61">
         <f t="shared" si="17"/>
@@ -18668,25 +18690,25 @@
       <c r="AK37" s="28"/>
       <c r="AL37" s="28"/>
       <c r="AM37" s="28"/>
-      <c r="AN37" s="60">
-        <f>IFERROR(VLOOKUP(AD37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE37,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO37" s="60">
-        <f>IFERROR(VLOOKUP(AF37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG37,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP37" s="60">
-        <f>IFERROR(VLOOKUP(AH37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI37,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ37" s="60">
-        <f>IFERROR(VLOOKUP(AJ37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK37,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR37" s="60">
-        <f>IFERROR(VLOOKUP(AL37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM37,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN37" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE37,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO37" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG37,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP37" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI37,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ37" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK37,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR37" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL37,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM37,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS37" s="61">
         <f t="shared" si="17"/>
@@ -18853,25 +18875,25 @@
       <c r="AK38" s="28"/>
       <c r="AL38" s="28"/>
       <c r="AM38" s="28"/>
-      <c r="AN38" s="60">
-        <f>IFERROR(VLOOKUP(AD38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE38,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO38" s="60">
-        <f>IFERROR(VLOOKUP(AF38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG38,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP38" s="60">
-        <f>IFERROR(VLOOKUP(AH38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI38,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ38" s="60">
-        <f>IFERROR(VLOOKUP(AJ38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK38,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR38" s="60">
-        <f>IFERROR(VLOOKUP(AL38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM38,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN38" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE38,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO38" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG38,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP38" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI38,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ38" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK38,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR38" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL38,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM38,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS38" s="61">
         <f t="shared" si="17"/>
@@ -19038,25 +19060,25 @@
       <c r="AK39" s="28"/>
       <c r="AL39" s="28"/>
       <c r="AM39" s="28"/>
-      <c r="AN39" s="60">
-        <f>IFERROR(VLOOKUP(AD39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE39,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO39" s="60">
-        <f>IFERROR(VLOOKUP(AF39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG39,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP39" s="60">
-        <f>IFERROR(VLOOKUP(AH39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI39,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ39" s="60">
-        <f>IFERROR(VLOOKUP(AJ39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK39,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR39" s="60">
-        <f>IFERROR(VLOOKUP(AL39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM39,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN39" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE39,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO39" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG39,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP39" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI39,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ39" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK39,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR39" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL39,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM39,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS39" s="61">
         <f t="shared" si="17"/>
@@ -19223,25 +19245,25 @@
       <c r="AK40" s="28"/>
       <c r="AL40" s="28"/>
       <c r="AM40" s="28"/>
-      <c r="AN40" s="60">
-        <f>IFERROR(VLOOKUP(AD40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE40,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO40" s="60">
-        <f>IFERROR(VLOOKUP(AF40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG40,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP40" s="60">
-        <f>IFERROR(VLOOKUP(AH40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI40,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ40" s="60">
-        <f>IFERROR(VLOOKUP(AJ40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK40,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR40" s="60">
-        <f>IFERROR(VLOOKUP(AL40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM40,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN40" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE40,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO40" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG40,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP40" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI40,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ40" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK40,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR40" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL40,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM40,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS40" s="61">
         <f t="shared" si="17"/>
@@ -19408,25 +19430,25 @@
       <c r="AK41" s="28"/>
       <c r="AL41" s="28"/>
       <c r="AM41" s="28"/>
-      <c r="AN41" s="60">
-        <f>IFERROR(VLOOKUP(AD41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE41,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO41" s="60">
-        <f>IFERROR(VLOOKUP(AF41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG41,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP41" s="60">
-        <f>IFERROR(VLOOKUP(AH41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI41,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ41" s="60">
-        <f>IFERROR(VLOOKUP(AJ41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK41,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR41" s="60">
-        <f>IFERROR(VLOOKUP(AL41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM41,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN41" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE41,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO41" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG41,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP41" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI41,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ41" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK41,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR41" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL41,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM41,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS41" s="61">
         <f t="shared" si="17"/>
@@ -19593,25 +19615,25 @@
       <c r="AK42" s="28"/>
       <c r="AL42" s="28"/>
       <c r="AM42" s="28"/>
-      <c r="AN42" s="60">
-        <f>IFERROR(VLOOKUP(AD42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE42,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO42" s="60">
-        <f>IFERROR(VLOOKUP(AF42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG42,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP42" s="60">
-        <f>IFERROR(VLOOKUP(AH42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI42,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ42" s="60">
-        <f>IFERROR(VLOOKUP(AJ42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK42,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR42" s="60">
-        <f>IFERROR(VLOOKUP(AL42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM42,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN42" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE42,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO42" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG42,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP42" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI42,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ42" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK42,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR42" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL42,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM42,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS42" s="61">
         <f t="shared" si="17"/>
@@ -19778,25 +19800,25 @@
       <c r="AK43" s="28"/>
       <c r="AL43" s="28"/>
       <c r="AM43" s="28"/>
-      <c r="AN43" s="60">
-        <f>IFERROR(VLOOKUP(AD43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE43,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO43" s="60">
-        <f>IFERROR(VLOOKUP(AF43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG43,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP43" s="60">
-        <f>IFERROR(VLOOKUP(AH43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI43,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ43" s="60">
-        <f>IFERROR(VLOOKUP(AJ43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK43,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR43" s="60">
-        <f>IFERROR(VLOOKUP(AL43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM43,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN43" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE43,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO43" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG43,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP43" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI43,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ43" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK43,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR43" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL43,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM43,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS43" s="61">
         <f t="shared" si="17"/>
@@ -19963,25 +19985,25 @@
       <c r="AK44" s="28"/>
       <c r="AL44" s="28"/>
       <c r="AM44" s="28"/>
-      <c r="AN44" s="60">
-        <f>IFERROR(VLOOKUP(AD44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE44,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO44" s="60">
-        <f>IFERROR(VLOOKUP(AF44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG44,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP44" s="60">
-        <f>IFERROR(VLOOKUP(AH44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI44,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ44" s="60">
-        <f>IFERROR(VLOOKUP(AJ44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK44,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR44" s="60">
-        <f>IFERROR(VLOOKUP(AL44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM44,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN44" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE44,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO44" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG44,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP44" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI44,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ44" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK44,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR44" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL44,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM44,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS44" s="61">
         <f t="shared" si="17"/>
@@ -20148,25 +20170,25 @@
       <c r="AK45" s="28"/>
       <c r="AL45" s="28"/>
       <c r="AM45" s="28"/>
-      <c r="AN45" s="60">
-        <f>IFERROR(VLOOKUP(AD45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE45,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO45" s="60">
-        <f>IFERROR(VLOOKUP(AF45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG45,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP45" s="60">
-        <f>IFERROR(VLOOKUP(AH45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI45,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ45" s="60">
-        <f>IFERROR(VLOOKUP(AJ45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK45,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR45" s="60">
-        <f>IFERROR(VLOOKUP(AL45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM45,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN45" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE45,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO45" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG45,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP45" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI45,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ45" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK45,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR45" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL45,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM45,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS45" s="61">
         <f t="shared" si="17"/>
@@ -20333,25 +20355,25 @@
       <c r="AK46" s="28"/>
       <c r="AL46" s="28"/>
       <c r="AM46" s="28"/>
-      <c r="AN46" s="60">
-        <f>IFERROR(VLOOKUP(AD46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE46,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO46" s="60">
-        <f>IFERROR(VLOOKUP(AF46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG46,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP46" s="60">
-        <f>IFERROR(VLOOKUP(AH46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI46,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ46" s="60">
-        <f>IFERROR(VLOOKUP(AJ46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK46,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR46" s="60">
-        <f>IFERROR(VLOOKUP(AL46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM46,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN46" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE46,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO46" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG46,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP46" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI46,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ46" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK46,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR46" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL46,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM46,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS46" s="61">
         <f t="shared" si="17"/>
@@ -20518,25 +20540,25 @@
       <c r="AK47" s="28"/>
       <c r="AL47" s="28"/>
       <c r="AM47" s="28"/>
-      <c r="AN47" s="60">
-        <f>IFERROR(VLOOKUP(AD47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE47,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO47" s="60">
-        <f>IFERROR(VLOOKUP(AF47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG47,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP47" s="60">
-        <f>IFERROR(VLOOKUP(AH47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI47,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ47" s="60">
-        <f>IFERROR(VLOOKUP(AJ47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK47,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR47" s="60">
-        <f>IFERROR(VLOOKUP(AL47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM47,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN47" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE47,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO47" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG47,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP47" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI47,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ47" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK47,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR47" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL47,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM47,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS47" s="61">
         <f t="shared" si="17"/>
@@ -20703,25 +20725,25 @@
       <c r="AK48" s="28"/>
       <c r="AL48" s="28"/>
       <c r="AM48" s="28"/>
-      <c r="AN48" s="60">
-        <f>IFERROR(VLOOKUP(AD48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE48,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO48" s="60">
-        <f>IFERROR(VLOOKUP(AF48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG48,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP48" s="60">
-        <f>IFERROR(VLOOKUP(AH48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI48,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ48" s="60">
-        <f>IFERROR(VLOOKUP(AJ48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK48,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR48" s="60">
-        <f>IFERROR(VLOOKUP(AL48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM48,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN48" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE48,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO48" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG48,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP48" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI48,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ48" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK48,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR48" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL48,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM48,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS48" s="61">
         <f t="shared" si="17"/>
@@ -20888,25 +20910,25 @@
       <c r="AK49" s="28"/>
       <c r="AL49" s="28"/>
       <c r="AM49" s="28"/>
-      <c r="AN49" s="60">
-        <f>IFERROR(VLOOKUP(AD49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE49,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO49" s="60">
-        <f>IFERROR(VLOOKUP(AF49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG49,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP49" s="60">
-        <f>IFERROR(VLOOKUP(AH49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI49,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ49" s="60">
-        <f>IFERROR(VLOOKUP(AJ49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK49,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR49" s="60">
-        <f>IFERROR(VLOOKUP(AL49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM49,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN49" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE49,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO49" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG49,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP49" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI49,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ49" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK49,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR49" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL49,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM49,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS49" s="61">
         <f t="shared" si="17"/>
@@ -21073,25 +21095,25 @@
       <c r="AK50" s="28"/>
       <c r="AL50" s="28"/>
       <c r="AM50" s="28"/>
-      <c r="AN50" s="60">
-        <f>IFERROR(VLOOKUP(AD50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE50,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AO50" s="60">
-        <f>IFERROR(VLOOKUP(AF50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG50,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AP50" s="60">
-        <f>IFERROR(VLOOKUP(AH50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI50,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AQ50" s="60">
-        <f>IFERROR(VLOOKUP(AJ50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK50,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="AR50" s="60">
-        <f>IFERROR(VLOOKUP(AL50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM50,'RATE MASTER'!$A$26:$C$29,3,1),0),"")</f>
-        <v>4</v>
+      <c r="AN50" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AD50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AE50,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AO50" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AF50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AG50,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AP50" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AH50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AI50,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AQ50" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AJ50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AK50,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
+      </c>
+      <c r="AR50" s="60" t="str">
+        <f>IFERROR(VLOOKUP(AL50,'RATE MASTER'!$A:$G,7,0)+IFERROR(VLOOKUP(AM50,'RATE MASTER'!$K$7:$M$10,3,1),0),"")</f>
+        <v/>
       </c>
       <c r="AS50" s="61">
         <f t="shared" si="17"/>
@@ -21237,18 +21259,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="110" t="s">
         <v>329</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
@@ -21334,7 +21356,7 @@
         <f>'CBB+PP'!S7</f>
         <v>0</v>
       </c>
-      <c r="G8" s="110">
+      <c r="G8" s="88">
         <f>'CBB+PP'!U7</f>
         <v>0</v>
       </c>
@@ -21376,7 +21398,7 @@
         <f>'CBB+PP'!S8</f>
         <v>0</v>
       </c>
-      <c r="G9" s="111">
+      <c r="G9" s="89">
         <f>'CBB+PP'!U8</f>
         <v>0</v>
       </c>
@@ -21418,7 +21440,7 @@
         <f>'CBB+PP'!S9</f>
         <v>0</v>
       </c>
-      <c r="G10" s="110">
+      <c r="G10" s="88">
         <f>'CBB+PP'!U9</f>
         <v>0</v>
       </c>
@@ -21460,7 +21482,7 @@
         <f>'CBB+PP'!S10</f>
         <v>0</v>
       </c>
-      <c r="G11" s="111">
+      <c r="G11" s="89">
         <f>'CBB+PP'!U10</f>
         <v>0</v>
       </c>
@@ -21502,7 +21524,7 @@
         <f>'CBB+PP'!S11</f>
         <v>0</v>
       </c>
-      <c r="G12" s="110">
+      <c r="G12" s="88">
         <f>'CBB+PP'!U11</f>
         <v>0</v>
       </c>
@@ -21544,7 +21566,7 @@
         <f>'CBB+PP'!S12</f>
         <v>0</v>
       </c>
-      <c r="G13" s="111">
+      <c r="G13" s="89">
         <f>'CBB+PP'!U12</f>
         <v>0</v>
       </c>
@@ -21587,7 +21609,7 @@
         <f>'CBB+PP'!S13</f>
         <v>0</v>
       </c>
-      <c r="G14" s="110">
+      <c r="G14" s="88">
         <f>'CBB+PP'!U13</f>
         <v>0</v>
       </c>
@@ -21631,7 +21653,7 @@
         <f>'CBB+PP'!S14</f>
         <v>0</v>
       </c>
-      <c r="G15" s="111">
+      <c r="G15" s="89">
         <f>'CBB+PP'!U14</f>
         <v>0</v>
       </c>
@@ -21675,7 +21697,7 @@
         <f>'CBB+PP'!S15</f>
         <v>0</v>
       </c>
-      <c r="G16" s="110">
+      <c r="G16" s="88">
         <f>'CBB+PP'!U15</f>
         <v>0</v>
       </c>
@@ -21719,7 +21741,7 @@
         <f>'CBB+PP'!S16</f>
         <v>0</v>
       </c>
-      <c r="G17" s="111">
+      <c r="G17" s="89">
         <f>'CBB+PP'!U16</f>
         <v>0</v>
       </c>
@@ -21763,7 +21785,7 @@
         <f>'CBB+PP'!S17</f>
         <v>0</v>
       </c>
-      <c r="G18" s="110">
+      <c r="G18" s="88">
         <f>'CBB+PP'!U17</f>
         <v>0</v>
       </c>
@@ -21807,7 +21829,7 @@
         <f>'CBB+PP'!S18</f>
         <v>0</v>
       </c>
-      <c r="G19" s="111">
+      <c r="G19" s="89">
         <f>'CBB+PP'!U18</f>
         <v>0</v>
       </c>
@@ -21851,7 +21873,7 @@
         <f>'CBB+PP'!S19</f>
         <v>0</v>
       </c>
-      <c r="G20" s="110">
+      <c r="G20" s="88">
         <f>'CBB+PP'!U19</f>
         <v>0</v>
       </c>
@@ -21895,7 +21917,7 @@
         <f>'CBB+PP'!S20</f>
         <v>0</v>
       </c>
-      <c r="G21" s="111">
+      <c r="G21" s="89">
         <f>'CBB+PP'!U20</f>
         <v>0</v>
       </c>
@@ -21937,7 +21959,7 @@
         <f>'CBB+PP'!S21</f>
         <v>0</v>
       </c>
-      <c r="G22" s="110">
+      <c r="G22" s="88">
         <f>'CBB+PP'!U21</f>
         <v>0</v>
       </c>
@@ -21979,7 +22001,7 @@
         <f>'CBB+PP'!S22</f>
         <v>0</v>
       </c>
-      <c r="G23" s="111">
+      <c r="G23" s="89">
         <f>'CBB+PP'!U22</f>
         <v>0</v>
       </c>
@@ -22021,7 +22043,7 @@
         <f>'CBB+PP'!S23</f>
         <v>0</v>
       </c>
-      <c r="G24" s="110">
+      <c r="G24" s="88">
         <f>'CBB+PP'!U23</f>
         <v>0</v>
       </c>
@@ -22063,7 +22085,7 @@
         <f>'CBB+PP'!S24</f>
         <v>0</v>
       </c>
-      <c r="G25" s="111">
+      <c r="G25" s="89">
         <f>'CBB+PP'!U24</f>
         <v>0</v>
       </c>
@@ -22105,7 +22127,7 @@
         <f>'CBB+PP'!S25</f>
         <v>0</v>
       </c>
-      <c r="G26" s="110">
+      <c r="G26" s="88">
         <f>'CBB+PP'!U25</f>
         <v>0</v>
       </c>
@@ -22147,7 +22169,7 @@
         <f>'CBB+PP'!S26</f>
         <v>0</v>
       </c>
-      <c r="G27" s="111">
+      <c r="G27" s="89">
         <f>'CBB+PP'!U26</f>
         <v>0</v>
       </c>
@@ -22189,7 +22211,7 @@
         <f>'CBB+PP'!S27</f>
         <v>0</v>
       </c>
-      <c r="G28" s="110">
+      <c r="G28" s="88">
         <f>'CBB+PP'!U27</f>
         <v>0</v>
       </c>
@@ -22231,7 +22253,7 @@
         <f>'CBB+PP'!S28</f>
         <v>0</v>
       </c>
-      <c r="G29" s="111">
+      <c r="G29" s="89">
         <f>'CBB+PP'!U28</f>
         <v>0</v>
       </c>
@@ -22273,7 +22295,7 @@
         <f>'CBB+PP'!S29</f>
         <v>0</v>
       </c>
-      <c r="G30" s="110">
+      <c r="G30" s="88">
         <f>'CBB+PP'!U29</f>
         <v>0</v>
       </c>
@@ -22315,7 +22337,7 @@
         <f>'CBB+PP'!S30</f>
         <v>0</v>
       </c>
-      <c r="G31" s="111">
+      <c r="G31" s="89">
         <f>'CBB+PP'!U30</f>
         <v>0</v>
       </c>
@@ -22357,7 +22379,7 @@
         <f>'CBB+PP'!S31</f>
         <v>0</v>
       </c>
-      <c r="G32" s="110">
+      <c r="G32" s="88">
         <f>'CBB+PP'!U31</f>
         <v>0</v>
       </c>
@@ -22399,7 +22421,7 @@
         <f>'CBB+PP'!S32</f>
         <v>0</v>
       </c>
-      <c r="G33" s="111">
+      <c r="G33" s="89">
         <f>'CBB+PP'!U32</f>
         <v>0</v>
       </c>
@@ -22441,7 +22463,7 @@
         <f>'CBB+PP'!S33</f>
         <v>0</v>
       </c>
-      <c r="G34" s="110">
+      <c r="G34" s="88">
         <f>'CBB+PP'!U33</f>
         <v>0</v>
       </c>
@@ -22483,7 +22505,7 @@
         <f>'CBB+PP'!S34</f>
         <v>0</v>
       </c>
-      <c r="G35" s="111">
+      <c r="G35" s="89">
         <f>'CBB+PP'!U34</f>
         <v>0</v>
       </c>
@@ -22525,7 +22547,7 @@
         <f>'CBB+PP'!S35</f>
         <v>0</v>
       </c>
-      <c r="G36" s="110">
+      <c r="G36" s="88">
         <f>'CBB+PP'!U35</f>
         <v>0</v>
       </c>
@@ -22567,7 +22589,7 @@
         <f>'CBB+PP'!S36</f>
         <v>0</v>
       </c>
-      <c r="G37" s="111">
+      <c r="G37" s="89">
         <f>'CBB+PP'!U36</f>
         <v>0</v>
       </c>
@@ -22585,116 +22607,116 @@
       </c>
     </row>
     <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="109" t="s">
+      <c r="A39" s="111" t="s">
         <v>336</v>
       </c>
-      <c r="B39" s="99"/>
-      <c r="C39" s="99"/>
-      <c r="D39" s="99"/>
-      <c r="E39" s="99"/>
-      <c r="F39" s="99"/>
-      <c r="G39" s="99"/>
-      <c r="H39" s="99"/>
-      <c r="I39" s="99"/>
-      <c r="J39" s="99"/>
+      <c r="B39" s="101"/>
+      <c r="C39" s="101"/>
+      <c r="D39" s="101"/>
+      <c r="E39" s="101"/>
+      <c r="F39" s="101"/>
+      <c r="G39" s="101"/>
+      <c r="H39" s="101"/>
+      <c r="I39" s="101"/>
+      <c r="J39" s="101"/>
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="107" t="s">
+      <c r="A40" s="109" t="s">
         <v>337</v>
       </c>
-      <c r="B40" s="99"/>
-      <c r="C40" s="99"/>
-      <c r="D40" s="99"/>
-      <c r="E40" s="99"/>
-      <c r="F40" s="99"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="99"/>
-      <c r="I40" s="99"/>
-      <c r="J40" s="99"/>
+      <c r="B40" s="101"/>
+      <c r="C40" s="101"/>
+      <c r="D40" s="101"/>
+      <c r="E40" s="101"/>
+      <c r="F40" s="101"/>
+      <c r="G40" s="101"/>
+      <c r="H40" s="101"/>
+      <c r="I40" s="101"/>
+      <c r="J40" s="101"/>
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="107" t="s">
+      <c r="A41" s="109" t="s">
         <v>338</v>
       </c>
-      <c r="B41" s="99"/>
-      <c r="C41" s="99"/>
-      <c r="D41" s="99"/>
-      <c r="E41" s="99"/>
-      <c r="F41" s="99"/>
-      <c r="G41" s="99"/>
-      <c r="H41" s="99"/>
-      <c r="I41" s="99"/>
-      <c r="J41" s="99"/>
+      <c r="B41" s="101"/>
+      <c r="C41" s="101"/>
+      <c r="D41" s="101"/>
+      <c r="E41" s="101"/>
+      <c r="F41" s="101"/>
+      <c r="G41" s="101"/>
+      <c r="H41" s="101"/>
+      <c r="I41" s="101"/>
+      <c r="J41" s="101"/>
     </row>
     <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="107" t="s">
+      <c r="A42" s="109" t="s">
         <v>339</v>
       </c>
-      <c r="B42" s="99"/>
-      <c r="C42" s="99"/>
-      <c r="D42" s="99"/>
-      <c r="E42" s="99"/>
-      <c r="F42" s="99"/>
-      <c r="G42" s="99"/>
-      <c r="H42" s="99"/>
-      <c r="I42" s="99"/>
-      <c r="J42" s="99"/>
+      <c r="B42" s="101"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="101"/>
+      <c r="E42" s="101"/>
+      <c r="F42" s="101"/>
+      <c r="G42" s="101"/>
+      <c r="H42" s="101"/>
+      <c r="I42" s="101"/>
+      <c r="J42" s="101"/>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="107" t="s">
+      <c r="A43" s="109" t="s">
         <v>340</v>
       </c>
-      <c r="B43" s="99"/>
-      <c r="C43" s="99"/>
-      <c r="D43" s="99"/>
-      <c r="E43" s="99"/>
-      <c r="F43" s="99"/>
-      <c r="G43" s="99"/>
-      <c r="H43" s="99"/>
-      <c r="I43" s="99"/>
-      <c r="J43" s="99"/>
+      <c r="B43" s="101"/>
+      <c r="C43" s="101"/>
+      <c r="D43" s="101"/>
+      <c r="E43" s="101"/>
+      <c r="F43" s="101"/>
+      <c r="G43" s="101"/>
+      <c r="H43" s="101"/>
+      <c r="I43" s="101"/>
+      <c r="J43" s="101"/>
     </row>
     <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="107" t="s">
+      <c r="A44" s="109" t="s">
         <v>341</v>
       </c>
-      <c r="B44" s="99"/>
-      <c r="C44" s="99"/>
-      <c r="D44" s="99"/>
-      <c r="E44" s="99"/>
-      <c r="F44" s="99"/>
-      <c r="G44" s="99"/>
-      <c r="H44" s="99"/>
-      <c r="I44" s="99"/>
-      <c r="J44" s="99"/>
+      <c r="B44" s="101"/>
+      <c r="C44" s="101"/>
+      <c r="D44" s="101"/>
+      <c r="E44" s="101"/>
+      <c r="F44" s="101"/>
+      <c r="G44" s="101"/>
+      <c r="H44" s="101"/>
+      <c r="I44" s="101"/>
+      <c r="J44" s="101"/>
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" s="107" t="s">
+      <c r="A45" s="109" t="s">
         <v>342</v>
       </c>
-      <c r="B45" s="99"/>
-      <c r="C45" s="99"/>
-      <c r="D45" s="99"/>
-      <c r="E45" s="99"/>
-      <c r="F45" s="99"/>
-      <c r="G45" s="99"/>
-      <c r="H45" s="99"/>
-      <c r="I45" s="99"/>
-      <c r="J45" s="99"/>
+      <c r="B45" s="101"/>
+      <c r="C45" s="101"/>
+      <c r="D45" s="101"/>
+      <c r="E45" s="101"/>
+      <c r="F45" s="101"/>
+      <c r="G45" s="101"/>
+      <c r="H45" s="101"/>
+      <c r="I45" s="101"/>
+      <c r="J45" s="101"/>
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="107" t="s">
+      <c r="A46" s="109" t="s">
         <v>343</v>
       </c>
-      <c r="B46" s="99"/>
-      <c r="C46" s="99"/>
-      <c r="D46" s="99"/>
-      <c r="E46" s="99"/>
-      <c r="F46" s="99"/>
-      <c r="G46" s="99"/>
-      <c r="H46" s="99"/>
-      <c r="I46" s="99"/>
-      <c r="J46" s="99"/>
+      <c r="B46" s="101"/>
+      <c r="C46" s="101"/>
+      <c r="D46" s="101"/>
+      <c r="E46" s="101"/>
+      <c r="F46" s="101"/>
+      <c r="G46" s="101"/>
+      <c r="H46" s="101"/>
+      <c r="I46" s="101"/>
+      <c r="J46" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>